<commit_message>
data: generate 07_Coordinates via OSM Nominatim
Geocodes all 20 places with the Nominatim search API (rate-limited to
1 req/sec per its usage policy). Four places needed a corrected query
or a direct override because their common tourist name doesn't match
Nominatim's indexed OSM name (e.g. San Thome Basilica -> Santhome
Cathedral, DakshinaChitra found via Overpass name search since it
isn't indexed by Nominatim at all). Each lookup is logged to
evidence_log.jsonl for the 08_Evidence table.
</commit_message>
<xml_diff>
--- a/data/BayesTrip_Data.xlsx
+++ b/data/BayesTrip_Data.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="01_Place_Master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="07_Coordinates" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -986,4 +987,505 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>place_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>lng</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Marina Beach</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>13.0532752</v>
+      </c>
+      <c r="D2" t="n">
+        <v>80.28331059999999</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fort St. George</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>13.0798617</v>
+      </c>
+      <c r="D3" t="n">
+        <v>80.2846692</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kapaleeshwarar Temple</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>13.0334336</v>
+      </c>
+      <c r="D4" t="n">
+        <v>80.26869600000001</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>San Thome Basilica</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>13.0335889</v>
+      </c>
+      <c r="D5" t="n">
+        <v>80.2777851</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Government Museum, Chennai</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>13.0712808</v>
+      </c>
+      <c r="D6" t="n">
+        <v>80.25704330000001</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Guindy National Park</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>13.000005</v>
+      </c>
+      <c r="D7" t="n">
+        <v>80.22804480000001</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Arignar Anna Zoological Park (Vandalur Zoo)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>12.8800708</v>
+      </c>
+      <c r="D8" t="n">
+        <v>80.08234539999999</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Valluvar Kottam</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>13.0540763</v>
+      </c>
+      <c r="D9" t="n">
+        <v>80.2418275</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Birla Planetarium</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>13.0119591</v>
+      </c>
+      <c r="D10" t="n">
+        <v>80.2440161</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Semmozhi Poonga</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>13.0506767</v>
+      </c>
+      <c r="D11" t="n">
+        <v>80.2514735</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Elliot's Beach</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>12.9969493</v>
+      </c>
+      <c r="D12" t="n">
+        <v>80.27087059999999</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Besant Nagar Beach</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>12.9978811</v>
+      </c>
+      <c r="D13" t="n">
+        <v>80.2718515</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DakshinaChitra</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>12.822513</v>
+      </c>
+      <c r="D14" t="n">
+        <v>80.2435254</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>OSM Overpass (name-substring search; not indexed by Nominatim)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Cholamandal Artists' Village</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>12.9224139</v>
+      </c>
+      <c r="D15" t="n">
+        <v>80.2522779</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Vivekananda House</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>13.0495712</v>
+      </c>
+      <c r="D16" t="n">
+        <v>80.2802712</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Thousand Lights Mosque</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>13.0550988</v>
+      </c>
+      <c r="D17" t="n">
+        <v>80.255239</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Parthasarathy Temple</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>13.0538288</v>
+      </c>
+      <c r="D18" t="n">
+        <v>80.2778941</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Vadapalani Murugan Temple</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>13.0529847</v>
+      </c>
+      <c r="D19" t="n">
+        <v>80.21426409999999</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Express Avenue</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>13.0588206</v>
+      </c>
+      <c r="D20" t="n">
+        <v>80.2641028</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>P20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MGM Dizzee World</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>12.8258571</v>
+      </c>
+      <c r="D21" t="n">
+        <v>80.2452821</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>OSM Nominatim</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
data: generate 04_HMM_Initial via OSRM travel time
Computes pi_i = 1/travel_time from Chennai Central to each place using
the OSRM public routing table service, normalized to sum to 1.
Deterministic, no LLM judgment.
</commit_message>
<xml_diff>
--- a/data/BayesTrip_Data.xlsx
+++ b/data/BayesTrip_Data.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="01_Place_Master" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="07_Coordinates" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="04_HMM_Initial" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1488,4 +1489,465 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>place_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>travel_time_seconds</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>raw_score</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>pi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Marina Beach</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>313.5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.003189792663476874</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.07560111097594464</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fort St. George</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>162.7</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.006146281499692687</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.1456727000058921</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kapaleeshwarar Temple</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>536.3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.001864628006712661</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.04419345196897007</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>San Thome Basilica</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>451.4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.002215330084182543</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.05250542377261553</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Government Museum, Chennai</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>291</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.003436426116838488</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.08144655770088882</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Guindy National Park</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1129.9</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.0008850340738118417</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.02097614681915094</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Arignar Anna Zoological Park (Vandalur Zoo)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2185.4</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.0004575821359934108</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.01084513054404624</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Valluvar Kottam</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>463.2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.002158894645941278</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.0511678503690817</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Birla Planetarium</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>924.1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.001082133968185261</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.02564760122384876</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Semmozhi Poonga</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>398.8</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.002507522567703109</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.05943066271554324</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Elliot's Beach</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>942.3</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.001061233152923697</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.02515223208209556</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Besant Nagar Beach</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>951.4</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.001051082615093546</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.02491165470985773</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DakshinaChitra</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2010.7</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.0004973392350922564</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.01178741149398649</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Cholamandal Artists' Village</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1372</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.0007288629737609329</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.01727474365230222</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Vivekananda House</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>323.7</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.003089280197713933</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.07321887022230042</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Thousand Lights Mosque</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>296.6</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.003371544167228591</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.07990879396816805</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Parthasarathy Temple</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>318.3</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.003141690229343387</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.07446103767187762</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Vadapalani Murugan Temple</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>735.7</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.001359249694168819</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.03221550671599652</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Express Avenue</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>287.3</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.003480682213713888</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.08249546916449232</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>P20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MGM Dizzee World</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2137.6</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.000467814371257485</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.01108764422294098</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
data: generate 05_HMM_Transition via OSRM travel time
Computes A_ij = 1/travel_time(i,j) for all 20x20 place pairs in a
single OSRM table request, each row normalized to sum to 1.
Deterministic, no LLM judgment.
</commit_message>
<xml_diff>
--- a/data/BayesTrip_Data.xlsx
+++ b/data/BayesTrip_Data.xlsx
@@ -10,6 +10,7 @@
     <sheet name="01_Place_Master" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="07_Coordinates" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="04_HMM_Initial" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="05_HMM_Transition" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1950,4 +1951,1570 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>from_place_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>from_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>P20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Marina Beach</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.06921107093768558</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.06260968889987915</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.08363109079911261</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.05044967268481613</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.02082086166198765</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.009445869758591149</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.0507720703286812</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.02646188757913808</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.06688059656068368</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.03006310740495241</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.02971033593185755</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.01255742615824914</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.01926290905037667</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.1558888059212147</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.06394772554858597</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.1399779192901308</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.02599612491837474</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.07056773511533088</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.011745101450352</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fort St. George</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.09487261675032413</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0556642743301005</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.06673727513770114</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.07394051212540154</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.02599282430608177</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.01334630695812448</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.05886349191773715</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.03140657113554399</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.06705452234017076</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.03246451819126585</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.03215837610262282</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.01533015508522997</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.02239667504260322</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.09200365531879937</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.08605888224911543</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.09350055118719804</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.03544584002173733</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.08833712763743531</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.01442582416280729</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kapaleeshwarar Temple</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0655870857272516</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.04288686920171556</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.2031780557853618</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0397091879573156</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.02630032553578173</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.009249208740518159</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.05287105833533403</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.03690043965485043</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.07218525177133675</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.04490192792096456</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.04406820512137105</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.01393947807537366</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.02371563339187872</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.1038856533428762</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.05470574298374862</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.07421933790372492</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.02568112643279899</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.05313118654362597</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.01288422557417166</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>San Thome Basilica</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.08014483026497554</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.04623889843200166</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.1527700573695644</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.03797174836353337</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.02211052246284202</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.008019543739837797</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.04958465943254734</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.03044658167489961</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.06929947673330189</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.03653706588796449</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.03591032262768085</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.01198290738079298</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.02002988766058741</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.1638041801718374</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.05141815426176704</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.0955387470109563</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.02332610034772216</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.05376919603156841</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.01109712014561932</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Government Museum, Chennai</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.07043898937378749</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.07439669678256217</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.05027594992093272</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.05724745820970006</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.02512067762195036</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.01211781750903794</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.07632994427960006</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.03068964254210412</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.08674563932386321</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.02746696619175635</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.02720092106951581</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.01278530385471788</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.01878925472010154</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.06851277572335149</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.1245383301404001</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.07525107580921703</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.03876708941870465</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.1113034204913332</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.01202204701736374</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Guindy National Park</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.04653491063506334</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.04632455694560299</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.05403702346178824</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.05381108102607675</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.05513531506148982</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.02629570716427528</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.07359930273602518</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.08378397536293312</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.06149496135928139</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.05751331919270144</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.0569744834008209</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.0296487092029024</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.04415840705970103</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.05076070053863266</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.06300013174774287</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0.05000389963605072</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.06443045258728294</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0.0547317928268394</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0.02776127005478947</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Arignar Anna Zoological Park (Vandalur Zoo)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0486478687439852</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.05058147870309573</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.04729197375365453</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.04820512587262191</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.05508608804510758</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.05068613454937136</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.05571248154130893</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.05117140151489909</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.0534291001186326</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.04998587125535054</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.04966286418933422</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.05907695113599609</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.06059611622833632</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.04917684895700165</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0.05308657496211586</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0.04911932977195649</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0.06161536551094457</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.05133224059941793</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0.05553618454686941</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Valluvar Kottam</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.05041353531546464</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.05193190640420579</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.0528124291563646</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.0577734690711328</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.1150421659740508</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.03609222201877147</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.01413192379367059</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.04039550605531444</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.1101849273193837</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.03223280003590295</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.03190969089256002</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.0147350411477013</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.02182611316475737</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.06391795541100175</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0.1045384965437242</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0.05731621961271465</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0.05988756955192472</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.07101646823306199</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.01384156029829223</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Birla Planetarium</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.04976262257548593</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.0413806669885002</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.06569863876379131</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.0619503476317988</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.04857574835933803</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.07191272515985427</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.0190766782685641</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.05833703706200109</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.06963241022564454</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.0691668055118359</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.06807671557391122</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.02621723175640388</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.04567452425328415</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.05879954461088457</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.05954778908101248</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0.0543973091231336</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0.04823597444149753</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0.05938585220180743</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.02417137841125097</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Semmozhi Poonga</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.04569158166885951</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.04373876030564454</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.04893132706836299</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.05611097038587047</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.07360695338726776</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.02274769069697452</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.008342189566886397</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.1647906815541118</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.02884166772436256</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.02507534664327499</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.02476164626596703</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.01008094335583166</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.01568956576120594</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.06602500547604259</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0.1884060825718036</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0.0556085875080717</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.03324404114777486</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0.07889453129156557</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0.009412427620121457</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Elliot's Beach</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.01495847738749461</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.01217976843658306</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.02059148959287547</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.02063983515269258</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.01179753971719406</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.01415441754278658</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.005319436196260419</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.01371448064808099</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.0199969846439998</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.01578491260227332</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.7469461911141101</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.008397587423062593</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.01582425467189959</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.01778443312176452</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0.01394372465110528</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0.0157479354058783</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0.01062403711447977</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0.01391316864383478</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.007681325933624065</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Besant Nagar Beach</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.01675290988342221</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.01367465541085158</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.02294671523568692</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.02299960660059187</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.01325002872597938</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.01586373746206899</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.006009069404147782</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.01537669289086512</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.02229594039658614</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.0176655020056296</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.7166728244604317</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.009460164908644847</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.01770891211294719</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.01986794014816023</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0.0156305315372139</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0.01762469853632312</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0.01194454707434053</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0.01559670328572059</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0.00865881992038837</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DakshinaChitra</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.02924563254341042</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.02684001019687128</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.03276717267221884</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.03279173293771347</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.02646039899840432</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.03092153624051011</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.02644194597943663</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.02882176131716934</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.03547086292077476</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.02985981078761497</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.04021067704126856</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.03978036064011348</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.071315337438458</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0.03119288192133508</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0.02843272589470092</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0.02983318380569148</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0.02698518770505326</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0.02840716328213888</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0.4042216176771162</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Cholamandal Artists' Village</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.04571061582774126</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.0404740990096175</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.05410414834223601</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.05416601428721349</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.0396812562943057</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.04959038624829524</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.03395343311635498</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.04476038787842203</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.06122014280060943</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.0471093494822009</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.07538418612208719</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.07399824758847996</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.08309451038069494</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.05023767469663324</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.04389887485253281</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0.04704816383461916</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0.04077964482029867</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0.04384261828501568</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0.07094624613264174</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Vivekananda House</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.1425116888244712</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.05850834975749344</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.05872681270635033</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.08560573490000402</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.04489081220366064</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.01682314179627655</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.007203913650604102</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.04783223395988612</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.02169938420079118</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.06381748072036447</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.02496525111585975</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.02464167358394931</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.009822254469905081</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0.01541009978025368</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0.06570800996312499</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0.2081939713994081</v>
+      </c>
+      <c r="T16" t="n">
+        <v>0.02178408338364493</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0.07269293707265045</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0.009162166511301599</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Thousand Lights Mosque</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.05959836855911219</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.042425957279368</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.0477647574733679</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.05499754438293369</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.06873162503959952</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.02222869668567391</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.008357324015598298</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.1111835110934698</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.02951900071421844</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.1812443537003138</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.02509915033627652</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.02479343186745023</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.01025419228751775</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0.01586295533799098</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.07069913338996973</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0.08113522973356141</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0.03091833241223847</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0.1056053189747553</v>
+      </c>
+      <c r="V17" t="n">
+        <v>0.009581116716584116</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Parthasarathy Temple</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.1311697330414792</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.06284072984623164</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.06319960386699462</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.08068498928069497</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.05182772542900939</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.02005006980695061</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.008681823447107275</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.05504321520039034</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.02494543623982573</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.06620437092742162</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.02797938550439003</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.02764463345588892</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.01155366130367004</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0.01780097206785397</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.1582130038115057</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0.07414142526991928</v>
+      </c>
+      <c r="S18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0.02581523413940959</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0.08140343866259818</v>
+      </c>
+      <c r="V18" t="n">
+        <v>0.01080054869865888</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Vadapalani Murugan Temple</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.04934309455627826</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.04902303124023754</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.04956482087381316</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.05257203852569594</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.07295615571594165</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.04859689629375775</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.02109784610602655</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.1299321028573631</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.05297465408553707</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.07588633973130858</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.03806703992864262</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.03774664586339044</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.02037425665593218</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.02991180995858821</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.0560522915911245</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0.07904643328974967</v>
+      </c>
+      <c r="S19" t="n">
+        <v>0.0548101981030053</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" t="n">
+        <v>0.06288393452619069</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0.01916041009741679</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Express Avenue</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.06078522822502774</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.05828586248505749</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.04763489881548406</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.05513006972722394</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.1029827608294867</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.02270537000700366</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.00954710984315266</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.07517563060897711</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.02894071181036816</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.09677898005662605</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.02559378030527484</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.02532185572760058</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.0113206855781866</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.01698235802262148</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.06807335037881324</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0.1779177147718613</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0.07612555082727236</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0.03008067882203869</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" t="n">
+        <v>0.01061740315792329</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>P20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MGM Dizzee World</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.02851529464733541</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.02629525897776664</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.03172720334110696</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.03174944763209145</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.0259429868673647</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.03004942361258944</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.02592584920924119</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.02812566327429361</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.03416308368118846</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0.02907869883893503</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.03837167631301262</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.0379927885120516</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.426592940575536</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0.06417728747348082</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.03029685852474086</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0.02776747596784301</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0.02905430154941465</v>
+      </c>
+      <c r="T21" t="n">
+        <v>0.02642984008234891</v>
+      </c>
+      <c r="U21" t="n">
+        <v>0.02774392091965878</v>
+      </c>
+      <c r="V21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
data: generate 06_HMM_Emission from opening-hours research
Opening hours were researched per place (raw/opening_hours_research.json,
free text with sources) and hand-extracted into structured daily
intervals (raw/opening_hours.json). This step is the deterministic
scoring pass: fixed Morning/Afternoon/Evening slots, 1.0 if a slot is
fully covered by an open interval, 0.5 if partially covered, 0.02 floor
if not covered at all (never a hard 0, so Viterbi can't permanently
zero out a state), normalized per place to sum to 1.
</commit_message>
<xml_diff>
--- a/data/BayesTrip_Data.xlsx
+++ b/data/BayesTrip_Data.xlsx
@@ -12,6 +12,7 @@
     <sheet name="04_HMM_Initial" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="05_HMM_Transition" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="03_BN_CPT" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="06_HMM_Emission" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16479,4 +16480,2645 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>place_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>raw_score</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>probability</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>opening_hours_text</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Marina Beach</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>24/7 (open public beach, no gate/entry control)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>YoMetro / multiple travel guides</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://yometro.com/travel-guide/attraction-marina-beach-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Marina Beach</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>24/7 (open public beach, no gate/entry control)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>YoMetro / multiple travel guides</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://yometro.com/travel-guide/attraction-marina-beach-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Marina Beach</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>24/7 (open public beach, no gate/entry control)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>YoMetro / multiple travel guides</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://yometro.com/travel-guide/attraction-marina-beach-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Fort St. George</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.3289473684210527</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Mo-Th,Sa-Su 09:00-17:00; Fr off (fort/museum grounds); Fort St. George Museum specifically: Mo-Su 09:00-17:00; Fr off (per OSM/Overpass)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Chennai Tourism (chennaitourism.travel) and OSM/Overpass-provided data</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://chennaitourism.travel/fort-st-george-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fort St. George</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.6578947368421053</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Mo-Th,Sa-Su 09:00-17:00; Fr off (fort/museum grounds); Fort St. George Museum specifically: Mo-Su 09:00-17:00; Fr off (per OSM/Overpass)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Chennai Tourism (chennaitourism.travel) and OSM/Overpass-provided data</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://chennaitourism.travel/fort-st-george-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Fort St. George</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.0131578947368421</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Mo-Th,Sa-Su 09:00-17:00; Fr off (fort/museum grounds); Fort St. George Museum specifically: Mo-Su 09:00-17:00; Fr off (per OSM/Overpass)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Chennai Tourism (chennaitourism.travel) and OSM/Overpass-provided data</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://chennaitourism.travel/fort-st-george-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Kapaleeshwarar Temple</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Mo-Su 05:00-12:30,16:00-21:30 (most sources: open daily, no weekly closure); one source (Tamil Nadu Tourism) states closed Mondays with hours 05:00-12:00,17:00-21:00</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Multiple travel sites (ciplore.com, indianpanorama.in, ymetro.com) vs. tamilnadutourism.com</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.tamilnadutourism.com/chennai/temples/kapaleeshwarar-temple.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Kapaleeshwarar Temple</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Mo-Su 05:00-12:30,16:00-21:30 (most sources: open daily, no weekly closure); one source (Tamil Nadu Tourism) states closed Mondays with hours 05:00-12:00,17:00-21:00</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Multiple travel sites (ciplore.com, indianpanorama.in, ymetro.com) vs. tamilnadutourism.com</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.tamilnadutourism.com/chennai/temples/kapaleeshwarar-temple.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kapaleeshwarar Temple</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Mo-Su 05:00-12:30,16:00-21:30 (most sources: open daily, no weekly closure); one source (Tamil Nadu Tourism) states closed Mondays with hours 05:00-12:00,17:00-21:00</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Multiple travel sites (ciplore.com, indianpanorama.in, ymetro.com) vs. tamilnadutourism.com</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.tamilnadutourism.com/chennai/temples/kapaleeshwarar-temple.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>San Thome Basilica</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Mo-Su 05:00-21:00 (general church/visiting hours per trawell.in); Mass times: Mon-Sat 05:45,06:15,11:00,17:45,18:15; Sun 06:00,07:15,08:30,10:00,11:30,17:30,18:00</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>trawell.in</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.trawell.in/tamilnadu/chennai/san-thome-cathedral-basilica</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>San Thome Basilica</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Mo-Su 05:00-21:00 (general church/visiting hours per trawell.in); Mass times: Mon-Sat 05:45,06:15,11:00,17:45,18:15; Sun 06:00,07:15,08:30,10:00,11:30,17:30,18:00</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>trawell.in</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://www.trawell.in/tamilnadu/chennai/san-thome-cathedral-basilica</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>San Thome Basilica</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Mo-Su 05:00-21:00 (general church/visiting hours per trawell.in); Mass times: Mon-Sat 05:45,06:15,11:00,17:45,18:15; Sun 06:00,07:15,08:30,10:00,11:30,17:30,18:00</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>trawell.in</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://www.trawell.in/tamilnadu/chennai/san-thome-cathedral-basilica</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Government Museum, Chennai</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.3289473684210527</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Sa-Th 09:30-17:00 (sometimes cited as 09:30-17:30); Fr off</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>trawell.in</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://www.trawell.in/tamilnadu/chennai/govt-museum</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Government Museum, Chennai</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.6578947368421053</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Sa-Th 09:30-17:00 (sometimes cited as 09:30-17:30); Fr off</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>trawell.in</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://www.trawell.in/tamilnadu/chennai/govt-museum</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Government Museum, Chennai</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.0131578947368421</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Sa-Th 09:30-17:00 (sometimes cited as 09:30-17:30); Fr off</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>trawell.in</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://www.trawell.in/tamilnadu/chennai/govt-museum</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Guindy National Park</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>9:00 AM - 5:30 PM (Wikipedia states 9 AM - 6 PM); closed Tuesdays</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Guindy_National_Park</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Guindy National Park</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>9:00 AM - 5:30 PM (Wikipedia states 9 AM - 6 PM); closed Tuesdays</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Guindy_National_Park</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Guindy National Park</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>9:00 AM - 5:30 PM (Wikipedia states 9 AM - 6 PM); closed Tuesdays</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Guindy_National_Park</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Arignar Anna Zoological Park (Vandalur Zoo)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.3289473684210527</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>9:00 AM - 5:00 PM (Wikipedia states 8:30 AM - 5:30 PM); closed Tuesdays</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Arignar_Anna_Zoological_Park</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Arignar Anna Zoological Park (Vandalur Zoo)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.6578947368421053</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>9:00 AM - 5:00 PM (Wikipedia states 8:30 AM - 5:30 PM); closed Tuesdays</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Arignar_Anna_Zoological_Park</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Arignar Anna Zoological Park (Vandalur Zoo)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.0131578947368421</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>9:00 AM - 5:00 PM (Wikipedia states 8:30 AM - 5:30 PM); closed Tuesdays</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Arignar_Anna_Zoological_Park</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Valluvar Kottam</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>10:00 AM - 8:00 PM daily (some sources say 8:30 AM - 5:30 PM or 8 AM - 6 PM); no designated weekly closed day, closed on national holidays</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Chennai Tourism</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://chennaitourism.travel/valluvar-kottam-monument-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Valluvar Kottam</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>10:00 AM - 8:00 PM daily (some sources say 8:30 AM - 5:30 PM or 8 AM - 6 PM); no designated weekly closed day, closed on national holidays</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Chennai Tourism</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://chennaitourism.travel/valluvar-kottam-monument-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Valluvar Kottam</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>10:00 AM - 8:00 PM daily (some sources say 8:30 AM - 5:30 PM or 8 AM - 6 PM); no designated weekly closed day, closed on national holidays</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Chennai Tourism</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://chennaitourism.travel/valluvar-kottam-monument-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Birla Planetarium</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Open daily 10:00 AM - 5:45 PM, closed only on national holidays. English 3D/sky show timings: 10:45 AM, 1:15 PM, 3:45 PM. Tamil show timings: 12:00 PM, 2:30 PM, 4:30 PM. Saturday night sky observation show: 7:00 PM - 9:00 PM.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Birla_Planetarium,_Chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Birla Planetarium</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Open daily 10:00 AM - 5:45 PM, closed only on national holidays. English 3D/sky show timings: 10:45 AM, 1:15 PM, 3:45 PM. Tamil show timings: 12:00 PM, 2:30 PM, 4:30 PM. Saturday night sky observation show: 7:00 PM - 9:00 PM.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Birla_Planetarium,_Chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Birla Planetarium</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Open daily 10:00 AM - 5:45 PM, closed only on national holidays. English 3D/sky show timings: 10:45 AM, 1:15 PM, 3:45 PM. Tamil show timings: 12:00 PM, 2:30 PM, 4:30 PM. Saturday night sky observation show: 7:00 PM - 9:00 PM.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Birla_Planetarium,_Chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Semmozhi Poonga</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>10:00 AM - 7:30 PM (Wikipedia states 10 AM - 8 PM) for general visitors, all days except Tuesday. Separate early-morning walkers' slot: 6:00 AM - 8:00 AM (monthly pass holders only, Rs.150).</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Semmozhi_Poonga</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Semmozhi Poonga</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>10:00 AM - 7:30 PM (Wikipedia states 10 AM - 8 PM) for general visitors, all days except Tuesday. Separate early-morning walkers' slot: 6:00 AM - 8:00 AM (monthly pass holders only, Rs.150).</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Semmozhi_Poonga</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Semmozhi Poonga</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>10:00 AM - 7:30 PM (Wikipedia states 10 AM - 8 PM) for general visitors, all days except Tuesday. Separate early-morning walkers' slot: 6:00 AM - 8:00 AM (monthly pass holders only, Rs.150).</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Semmozhi_Poonga</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Elliot's Beach</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Open 24 hours, every day</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>YoMetro / myholidayhappiness travel guides</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://yometro.com/travel-guide/attraction-elliots-beach-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Elliot's Beach</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Open 24 hours, every day</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>YoMetro / myholidayhappiness travel guides</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://yometro.com/travel-guide/attraction-elliots-beach-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Elliot's Beach</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Open 24 hours, every day</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>YoMetro / myholidayhappiness travel guides</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://yometro.com/travel-guide/attraction-elliots-beach-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Besant Nagar Beach</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Open 24 hours, every day</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>myholidayhappiness / Rehlat travel guides</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>https://myholidayhappiness.com/place/tamilnadu/chennai/besant-nagar-beach</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Besant Nagar Beach</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Open 24 hours, every day</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>myholidayhappiness / Rehlat travel guides</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://myholidayhappiness.com/place/tamilnadu/chennai/besant-nagar-beach</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Besant Nagar Beach</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Open 24 hours, every day</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>myholidayhappiness / Rehlat travel guides</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://myholidayhappiness.com/place/tamilnadu/chennai/besant-nagar-beach</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>DakshinaChitra</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Weekdays 10:00 AM - 6:00 PM; Weekends 10:00 AM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>DakshinaChitra official website</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://www.dakshinachitra.net/visit-Dakshinachitra</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>DakshinaChitra</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Weekdays 10:00 AM - 6:00 PM; Weekends 10:00 AM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>DakshinaChitra official website</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://www.dakshinachitra.net/visit-Dakshinachitra</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>DakshinaChitra</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Weekdays 10:00 AM - 6:00 PM; Weekends 10:00 AM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>DakshinaChitra official website</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://www.dakshinachitra.net/visit-Dakshinachitra</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Cholamandal Artists' Village</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>9:30 AM - 6:30 PM, every day of the week</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Chennai Tourism (chennaitourism.travel), corroborated by Trawell and other travel guides</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://chennaitourism.travel/cholamandal-artists-village-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Cholamandal Artists' Village</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>9:30 AM - 6:30 PM, every day of the week</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Chennai Tourism (chennaitourism.travel), corroborated by Trawell and other travel guides</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://chennaitourism.travel/cholamandal-artists-village-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Cholamandal Artists' Village</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>9:30 AM - 6:30 PM, every day of the week</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Chennai Tourism (chennaitourism.travel), corroborated by Trawell and other travel guides</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://chennaitourism.travel/cholamandal-artists-village-chennai</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Vivekananda House</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>10:00 AM - 12:30 PM and 3:00 PM - 7:15 PM (split morning/evening sessions)</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>IndianHoliday / Chennai Tourism travel guides</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>https://www.indianholiday.com/tamil-nadu/chennai/historical-monuments/vivekananda-illam-chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Vivekananda House</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>10:00 AM - 12:30 PM and 3:00 PM - 7:15 PM (split morning/evening sessions)</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>IndianHoliday / Chennai Tourism travel guides</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>https://www.indianholiday.com/tamil-nadu/chennai/historical-monuments/vivekananda-illam-chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Vivekananda House</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>10:00 AM - 12:30 PM and 3:00 PM - 7:15 PM (split morning/evening sessions)</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>IndianHoliday / Chennai Tourism travel guides</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://www.indianholiday.com/tamil-nadu/chennai/historical-monuments/vivekananda-illam-chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Thousand Lights Mosque</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Daily 5:30 AM - 9:00 PM. No formal midday closure to visitors, but avoid the 5 daily prayer times (especially Friday Jumu'ah early afternoon) when access for non-worshippers may be restricted.</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Multiple travel sites (Yatra.com, Holidify, Trawell)</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>https://www.yatra.com/india-tourism/attractions-in-chennai/thousand-lights-mosque</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Thousand Lights Mosque</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Daily 5:30 AM - 9:00 PM. No formal midday closure to visitors, but avoid the 5 daily prayer times (especially Friday Jumu'ah early afternoon) when access for non-worshippers may be restricted.</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Multiple travel sites (Yatra.com, Holidify, Trawell)</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://www.yatra.com/india-tourism/attractions-in-chennai/thousand-lights-mosque</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Thousand Lights Mosque</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Daily 5:30 AM - 9:00 PM. No formal midday closure to visitors, but avoid the 5 daily prayer times (especially Friday Jumu'ah early afternoon) when access for non-worshippers may be restricted.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Multiple travel sites (Yatra.com, Holidify, Trawell)</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>https://www.yatra.com/india-tourism/attractions-in-chennai/thousand-lights-mosque</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Parthasarathy Temple</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Daily: morning 6:00 AM - 12:00/12:30 PM, closed midday, reopens evening 4:00 PM - 9:00 PM. Saturday differs: 5:30 AM - 12:00 PM and 4:00 PM - 10:00 PM.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>GoTirupati / Trawell / DarshansTime (temple info aggregators)</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>https://gotirupati.com/parthasarathy-temple-triplicane/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Parthasarathy Temple</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Daily: morning 6:00 AM - 12:00/12:30 PM, closed midday, reopens evening 4:00 PM - 9:00 PM. Saturday differs: 5:30 AM - 12:00 PM and 4:00 PM - 10:00 PM.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>GoTirupati / Trawell / DarshansTime (temple info aggregators)</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>https://gotirupati.com/parthasarathy-temple-triplicane/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Parthasarathy Temple</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Daily: morning 6:00 AM - 12:00/12:30 PM, closed midday, reopens evening 4:00 PM - 9:00 PM. Saturday differs: 5:30 AM - 12:00 PM and 4:00 PM - 10:00 PM.</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>GoTirupati / Trawell / DarshansTime (temple info aggregators)</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>https://gotirupati.com/parthasarathy-temple-triplicane/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Vadapalani Murugan Temple</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Daily: 5:00 AM - 12:30 PM, closed midday, reopens 4:00 PM - 9:00 PM. Same schedule Monday to Sunday; extended/continuous hours during festival days.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>GoTirupati / DarshansBooking (temple info aggregators)</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>https://gotirupati.com/vadapalani-temple-timings/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Vadapalani Murugan Temple</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Daily: 5:00 AM - 12:30 PM, closed midday, reopens 4:00 PM - 9:00 PM. Same schedule Monday to Sunday; extended/continuous hours during festival days.</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>GoTirupati / DarshansBooking (temple info aggregators)</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>https://gotirupati.com/vadapalani-temple-timings/</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Vadapalani Murugan Temple</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Daily: 5:00 AM - 12:30 PM, closed midday, reopens 4:00 PM - 9:00 PM. Same schedule Monday to Sunday; extended/continuous hours during festival days.</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>GoTirupati / DarshansBooking (temple info aggregators)</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>https://gotirupati.com/vadapalani-temple-timings/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Express Avenue</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Daily 10:00 AM - 10:00 PM, same hours every day of the week including weekends and public holidays.</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Holidify / Rehlat / malls.com (travel/mall aggregator sites)</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>https://www.holidify.com/places/chennai/express-avenue-sightseeing-121150.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Express Avenue</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Daily 10:00 AM - 10:00 PM, same hours every day of the week including weekends and public holidays.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Holidify / Rehlat / malls.com (travel/mall aggregator sites)</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>https://www.holidify.com/places/chennai/express-avenue-sightseeing-121150.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Express Avenue</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Daily 10:00 AM - 10:00 PM, same hours every day of the week including weekends and public holidays.</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Holidify / Rehlat / malls.com (travel/mall aggregator sites)</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>https://www.holidify.com/places/chennai/express-avenue-sightseeing-121150.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>P20</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>MGM Dizzee World</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Mo-Fr 10:30 AM - 6:00 PM; Sa-Su and Public Holidays 10:30 AM - 6:30 PM. Extended to ~7:30 PM during peak summer (mid-April to end May) and winter (mid-December to end January) seasons.</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Official site (mgmdizzeeworld.com) and NativePlanet</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>https://www.mgmdizzeeworld.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>P20</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>MGM Dizzee World</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>fully open</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Mo-Fr 10:30 AM - 6:00 PM; Sa-Su and Public Holidays 10:30 AM - 6:30 PM. Extended to ~7:30 PM during peak summer (mid-April to end May) and winter (mid-December to end January) seasons.</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Official site (mgmdizzeeworld.com) and NativePlanet</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>https://www.mgmdizzeeworld.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>P20</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>MGM Dizzee World</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Mo-Fr 10:30 AM - 6:00 PM; Sa-Su and Public Holidays 10:30 AM - 6:30 PM. Extended to ~7:30 PM during peak summer (mid-April to end May) and winter (mid-December to end January) seasons.</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Official site (mgmdizzeeworld.com) and NativePlanet</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>https://www.mgmdizzeeworld.com/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>